<commit_message>
fix: update team leader to Vo Ngoc Minh Quan across all documents, slides, scripts and app
</commit_message>
<xml_diff>
--- a/outputs/tables/MAS291_DeTai1_BangTinh_Va_DuLieu_TongHop.xlsx
+++ b/outputs/tables/MAS291_DeTai1_BangTinh_Va_DuLieu_TongHop.xlsx
@@ -748,7 +748,7 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Nhóm trưởng</t>
+          <t>Thành viên</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Quản lý tiến độ dự án, tổ chức phân công, xây dựng kiến trúc mã nguồn Python &amp; Streamlit, tổng hợp báo cáo (Câu 1, 2)</t>
+          <t>Thu thập dữ liệu khảo sát ẩn danh, kiểm tra tính hợp lệ, thiết kế quy chuẩn làm sạch dữ liệu và định dạng báo cáo (Câu 1, 2)</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Thu thập dữ liệu khảo sát ẩn danh, kiểm tra tính hợp lệ, viết module làm sạch dữ liệu và thống kê mô tả (Câu 1, 2, 3, 4)</t>
+          <t>Xử lý thống kê mô tả, tính toán độ tập trung, độ phân tán và vẽ biểu đồ phân phối Histogram &amp; Boxplot (Câu 3, 4)</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Thành viên</t>
+          <t>Nhóm trưởng</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Vẽ đồ thị phân phối Histogram, Boxplot, phân tích ngoại lệ 1.5 IQR, tính tương quan Pearson và vẽ Scatterplot (Câu 4, 5, 6, 7)</t>
+          <t>Nhóm trưởng: Quản lý tiến độ dự án, tổ chức phân công, xây dựng kiến trúc mã nguồn Python &amp; Streamlit, ước lượng tương quan Pearson &amp; OLS (Câu 5, 6, 7)</t>
         </is>
       </c>
     </row>

</xml_diff>